<commit_message>
Add sale edit, F11 save-close, line prices, and sales PDF report
Legacy 1.6.4: F11 saves without printing, Sales History Edit reopens a
sale for item/price changes with stock-safe update_invoice, Export PDF
for accounting reports, and product import templates include Date Stamp.

Co-authored-by: theprincesajjad <theprincesajjad@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/legacy/assets/product_import_template.xlsx
+++ b/legacy/assets/product_import_template.xlsx
@@ -417,14 +417,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,6 +455,16 @@
           <t>Price</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Date Stamp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -476,29 +488,70 @@
       <c r="E2" t="n">
         <v>699.99</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Laptops</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>60001</t>
+          <t>92001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Laptop Case</t>
+          <t>ThinkPad X1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>15.6 inch</t>
+          <t>16GB 512GB</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>15</v>
-      </c>
+        <v>899</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Laptops</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>110001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>iPhone 13</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>128GB Blue</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>499</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cell Phones</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>